<commit_message>
Refactor table styling and improve data fetching for agriculture reports
</commit_message>
<xml_diff>
--- a/agriculture 6.xlsx
+++ b/agriculture 6.xlsx
@@ -25,7 +25,7 @@
     <t xml:space="preserve">Year</t>
   </si>
   <si>
-    <t xml:space="preserve">AREA (Thousand Hectares</t>
+    <t xml:space="preserve">AREA (Thousand Hectares)</t>
   </si>
   <si>
     <t xml:space="preserve">Andhra Pradesh</t>
@@ -599,7 +599,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Y1048576"/>
-  <sheetFormatPr defaultColWidth="10.78515625" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.796875" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12.18"/>

</xml_diff>